<commit_message>
Pipeline OK: PDFs procesados, cronología normalizada y matriz CPP
</commit_message>
<xml_diff>
--- a/nicaragua/denuncia_maria_fatima/resultados/matriz_evidencia.xlsx
+++ b/nicaragua/denuncia_maria_fatima/resultados/matriz_evidencia.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,34 @@
           <t>Observaciones</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Indice Y Analisis.pdf</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REPORTE COMPLETO INDICE.pdf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>